<commit_message>
User Management Issue Solved
</commit_message>
<xml_diff>
--- a/locations.xlsx
+++ b/locations.xlsx
@@ -1096,7 +1096,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C104"/>
+  <dimension ref="A1:C138"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1175,12 +1175,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>AR</t>
+          <t>AP</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Itanagar</t>
+          <t>Tirupati</t>
         </is>
       </c>
     </row>
@@ -1192,12 +1192,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>AR</t>
+          <t>AP</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Naharlagun</t>
+          <t>Kurnool</t>
         </is>
       </c>
     </row>
@@ -1209,12 +1209,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>AS</t>
+          <t>AP</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Guwahati</t>
+          <t>Nellore</t>
         </is>
       </c>
     </row>
@@ -1226,12 +1226,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>AS</t>
+          <t>AP</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Dibrugarh</t>
+          <t>Rajahmundry</t>
         </is>
       </c>
     </row>
@@ -1243,12 +1243,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>AS</t>
+          <t>AR</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Silchar</t>
+          <t>Itanagar</t>
         </is>
       </c>
     </row>
@@ -1260,12 +1260,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>BR</t>
+          <t>AR</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Patna</t>
+          <t>Naharlagun</t>
         </is>
       </c>
     </row>
@@ -1277,12 +1277,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>BR</t>
+          <t>AR</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Gaya</t>
+          <t>Tawang</t>
         </is>
       </c>
     </row>
@@ -1294,12 +1294,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>BR</t>
+          <t>AR</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Muzaffarpur</t>
+          <t>Pasighat</t>
         </is>
       </c>
     </row>
@@ -1311,12 +1311,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>CG</t>
+          <t>AS</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Raipur</t>
+          <t>Guwahati</t>
         </is>
       </c>
     </row>
@@ -1328,12 +1328,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>CG</t>
+          <t>AS</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Bilaspur</t>
+          <t>Dibrugarh</t>
         </is>
       </c>
     </row>
@@ -1345,12 +1345,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>CG</t>
+          <t>AS</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Durg</t>
+          <t>Silchar</t>
         </is>
       </c>
     </row>
@@ -1362,12 +1362,12 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>GA</t>
+          <t>AS</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Panaji</t>
+          <t>Jorhat</t>
         </is>
       </c>
     </row>
@@ -1379,12 +1379,12 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>GA</t>
+          <t>AS</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Margao</t>
+          <t>Tezpur</t>
         </is>
       </c>
     </row>
@@ -1396,12 +1396,12 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>GA</t>
+          <t>BR</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Vasco da Gama</t>
+          <t>Patna</t>
         </is>
       </c>
     </row>
@@ -1413,12 +1413,12 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>GJ</t>
+          <t>BR</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Ahmedabad</t>
+          <t>Gaya</t>
         </is>
       </c>
     </row>
@@ -1430,12 +1430,12 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>GJ</t>
+          <t>BR</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Surat</t>
+          <t>Muzaffarpur</t>
         </is>
       </c>
     </row>
@@ -1447,12 +1447,12 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>GJ</t>
+          <t>BR</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Vadodara</t>
+          <t>Bhagalpur</t>
         </is>
       </c>
     </row>
@@ -1464,12 +1464,12 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>GJ</t>
+          <t>BR</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Rajkot</t>
+          <t>Darbhanga</t>
         </is>
       </c>
     </row>
@@ -1481,12 +1481,12 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>HR</t>
+          <t>CG</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Gurugram</t>
+          <t>Raipur</t>
         </is>
       </c>
     </row>
@@ -1498,12 +1498,12 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>HR</t>
+          <t>CG</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Faridabad</t>
+          <t>Bilaspur</t>
         </is>
       </c>
     </row>
@@ -1515,12 +1515,12 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>HR</t>
+          <t>CG</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Panipat</t>
+          <t>Durg</t>
         </is>
       </c>
     </row>
@@ -1532,12 +1532,12 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>CG</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Shimla</t>
+          <t>Korba</t>
         </is>
       </c>
     </row>
@@ -1549,12 +1549,12 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>CG</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Dharamshala</t>
+          <t>Jagdalpur</t>
         </is>
       </c>
     </row>
@@ -1566,12 +1566,12 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>HP</t>
+          <t>GA</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Solan</t>
+          <t>Panaji</t>
         </is>
       </c>
     </row>
@@ -1583,12 +1583,12 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>JH</t>
+          <t>GA</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Ranchi</t>
+          <t>Margao</t>
         </is>
       </c>
     </row>
@@ -1600,12 +1600,12 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>JH</t>
+          <t>GA</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Jamshedpur</t>
+          <t>Mapusa</t>
         </is>
       </c>
     </row>
@@ -1617,12 +1617,12 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>JH</t>
+          <t>GA</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Dhanbad</t>
+          <t>Vasco da Gama</t>
         </is>
       </c>
     </row>
@@ -1634,12 +1634,12 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>KA</t>
+          <t>GJ</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Bengaluru</t>
+          <t>Ahmedabad</t>
         </is>
       </c>
     </row>
@@ -1651,12 +1651,12 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>KA</t>
+          <t>GJ</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Mysuru</t>
+          <t>Surat</t>
         </is>
       </c>
     </row>
@@ -1668,12 +1668,12 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>KA</t>
+          <t>GJ</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Mangaluru</t>
+          <t>Vadodara</t>
         </is>
       </c>
     </row>
@@ -1685,12 +1685,12 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>KA</t>
+          <t>GJ</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Hubballi</t>
+          <t>Rajkot</t>
         </is>
       </c>
     </row>
@@ -1702,12 +1702,12 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>KL</t>
+          <t>GJ</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Thiruvananthapuram</t>
+          <t>Bhavnagar</t>
         </is>
       </c>
     </row>
@@ -1719,12 +1719,12 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>KL</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Kochi</t>
+          <t>Gurugram</t>
         </is>
       </c>
     </row>
@@ -1736,12 +1736,12 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>KL</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Kozhikode</t>
+          <t>Faridabad</t>
         </is>
       </c>
     </row>
@@ -1753,12 +1753,12 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>MP</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Bhopal</t>
+          <t>Panipat</t>
         </is>
       </c>
     </row>
@@ -1770,12 +1770,12 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>MP</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Indore</t>
+          <t>Ambala</t>
         </is>
       </c>
     </row>
@@ -1787,12 +1787,12 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>MP</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Jabalpur</t>
+          <t>Hisar</t>
         </is>
       </c>
     </row>
@@ -1804,12 +1804,12 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>MP</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Gwalior</t>
+          <t>Shimla</t>
         </is>
       </c>
     </row>
@@ -1821,12 +1821,12 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>MH</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Mumbai</t>
+          <t>Dharamshala</t>
         </is>
       </c>
     </row>
@@ -1838,12 +1838,12 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>MH</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Pune</t>
+          <t>Solan</t>
         </is>
       </c>
     </row>
@@ -1855,12 +1855,12 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>MH</t>
+          <t>HP</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Nagpur</t>
+          <t>Mandi</t>
         </is>
       </c>
     </row>
@@ -1872,12 +1872,12 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>MH</t>
+          <t>JH</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Nashik</t>
+          <t>Ranchi</t>
         </is>
       </c>
     </row>
@@ -1889,12 +1889,12 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>MH</t>
+          <t>JH</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Aurangabad</t>
+          <t>Jamshedpur</t>
         </is>
       </c>
     </row>
@@ -1906,12 +1906,12 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>MH</t>
+          <t>JH</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Kolhapur</t>
+          <t>Dhanbad</t>
         </is>
       </c>
     </row>
@@ -1923,12 +1923,12 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>MH</t>
+          <t>JH</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Solapur</t>
+          <t>Bokaro</t>
         </is>
       </c>
     </row>
@@ -1940,12 +1940,12 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>MH</t>
+          <t>KA</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Amravati</t>
+          <t>Bengaluru</t>
         </is>
       </c>
     </row>
@@ -1957,12 +1957,12 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>MN</t>
+          <t>KA</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Imphal</t>
+          <t>Mysuru</t>
         </is>
       </c>
     </row>
@@ -1974,12 +1974,12 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>ML</t>
+          <t>KA</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Shillong</t>
+          <t>Mangaluru</t>
         </is>
       </c>
     </row>
@@ -1991,12 +1991,12 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>ML</t>
+          <t>KA</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Tura</t>
+          <t>Hubballi</t>
         </is>
       </c>
     </row>
@@ -2008,12 +2008,12 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>MZ</t>
+          <t>KA</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Aizawl</t>
+          <t>Belagavi</t>
         </is>
       </c>
     </row>
@@ -2025,12 +2025,12 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>MZ</t>
+          <t>KL</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Lunglei</t>
+          <t>Thiruvananthapuram</t>
         </is>
       </c>
     </row>
@@ -2042,12 +2042,12 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>NL</t>
+          <t>KL</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Kohima</t>
+          <t>Kochi</t>
         </is>
       </c>
     </row>
@@ -2059,12 +2059,12 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>NL</t>
+          <t>KL</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Dimapur</t>
+          <t>Kozhikode</t>
         </is>
       </c>
     </row>
@@ -2076,12 +2076,12 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>OD</t>
+          <t>KL</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Bhubaneswar</t>
+          <t>Thrissur</t>
         </is>
       </c>
     </row>
@@ -2093,12 +2093,12 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>OD</t>
+          <t>MP</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Cuttack</t>
+          <t>Bhopal</t>
         </is>
       </c>
     </row>
@@ -2110,12 +2110,12 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>OD</t>
+          <t>MP</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Rourkela</t>
+          <t>Indore</t>
         </is>
       </c>
     </row>
@@ -2127,12 +2127,12 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>PB</t>
+          <t>MP</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Ludhiana</t>
+          <t>Gwalior</t>
         </is>
       </c>
     </row>
@@ -2144,12 +2144,12 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>PB</t>
+          <t>MP</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Amritsar</t>
+          <t>Jabalpur</t>
         </is>
       </c>
     </row>
@@ -2161,12 +2161,12 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>PB</t>
+          <t>MP</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Jalandhar</t>
+          <t>Ujjain</t>
         </is>
       </c>
     </row>
@@ -2178,12 +2178,12 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>RJ</t>
+          <t>MH</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Jaipur</t>
+          <t>Mumbai</t>
         </is>
       </c>
     </row>
@@ -2195,12 +2195,12 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>RJ</t>
+          <t>MH</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Jodhpur</t>
+          <t>Pune</t>
         </is>
       </c>
     </row>
@@ -2212,12 +2212,12 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>RJ</t>
+          <t>MH</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Udaipur</t>
+          <t>Nagpur</t>
         </is>
       </c>
     </row>
@@ -2229,12 +2229,12 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>RJ</t>
+          <t>MH</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Kota</t>
+          <t>Nashik</t>
         </is>
       </c>
     </row>
@@ -2246,12 +2246,12 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>SK</t>
+          <t>MH</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Gangtok</t>
+          <t>Thane</t>
         </is>
       </c>
     </row>
@@ -2263,12 +2263,12 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>SK</t>
+          <t>MH</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Namchi</t>
+          <t>Aurangabad</t>
         </is>
       </c>
     </row>
@@ -2280,12 +2280,12 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>TN</t>
+          <t>MN</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Chennai</t>
+          <t>Imphal</t>
         </is>
       </c>
     </row>
@@ -2297,12 +2297,12 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>TN</t>
+          <t>MN</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Coimbatore</t>
+          <t>Thoubal</t>
         </is>
       </c>
     </row>
@@ -2314,12 +2314,12 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>TN</t>
+          <t>MN</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Madurai</t>
+          <t>Bishnupur</t>
         </is>
       </c>
     </row>
@@ -2331,12 +2331,12 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>TN</t>
+          <t>ML</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Salem</t>
+          <t>Shillong</t>
         </is>
       </c>
     </row>
@@ -2348,12 +2348,12 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>TN</t>
+          <t>ML</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Tiruchirappalli</t>
+          <t>Tura</t>
         </is>
       </c>
     </row>
@@ -2365,12 +2365,12 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>TS</t>
+          <t>ML</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Hyderabad</t>
+          <t>Jowai</t>
         </is>
       </c>
     </row>
@@ -2382,12 +2382,12 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>TS</t>
+          <t>MZ</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Warangal</t>
+          <t>Aizawl</t>
         </is>
       </c>
     </row>
@@ -2399,12 +2399,12 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>TS</t>
+          <t>MZ</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Karimnagar</t>
+          <t>Lunglei</t>
         </is>
       </c>
     </row>
@@ -2416,12 +2416,12 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>TR</t>
+          <t>MZ</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Agartala</t>
+          <t>Champhai</t>
         </is>
       </c>
     </row>
@@ -2433,12 +2433,12 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>NL</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Lucknow</t>
+          <t>Kohima</t>
         </is>
       </c>
     </row>
@@ -2450,12 +2450,12 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>NL</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Kanpur</t>
+          <t>Dimapur</t>
         </is>
       </c>
     </row>
@@ -2467,12 +2467,12 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>NL</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Varanasi</t>
+          <t>Mokokchung</t>
         </is>
       </c>
     </row>
@@ -2484,12 +2484,12 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>OD</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Agra</t>
+          <t>Bhubaneswar</t>
         </is>
       </c>
     </row>
@@ -2501,12 +2501,12 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>OD</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Prayagraj</t>
+          <t>Cuttack</t>
         </is>
       </c>
     </row>
@@ -2518,12 +2518,12 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>OD</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Noida</t>
+          <t>Rourkela</t>
         </is>
       </c>
     </row>
@@ -2535,12 +2535,12 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>UK</t>
+          <t>OD</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Dehradun</t>
+          <t>Sambalpur</t>
         </is>
       </c>
     </row>
@@ -2552,12 +2552,12 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>UK</t>
+          <t>PB</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Haridwar</t>
+          <t>Ludhiana</t>
         </is>
       </c>
     </row>
@@ -2569,12 +2569,12 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>UK</t>
+          <t>PB</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Haldwani</t>
+          <t>Amritsar</t>
         </is>
       </c>
     </row>
@@ -2586,12 +2586,12 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>WB</t>
+          <t>PB</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Kolkata</t>
+          <t>Jalandhar</t>
         </is>
       </c>
     </row>
@@ -2603,12 +2603,12 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>WB</t>
+          <t>PB</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Howrah</t>
+          <t>Patiala</t>
         </is>
       </c>
     </row>
@@ -2620,12 +2620,12 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>WB</t>
+          <t>RJ</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Durgapur</t>
+          <t>Jaipur</t>
         </is>
       </c>
     </row>
@@ -2637,12 +2637,12 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>WB</t>
+          <t>RJ</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Siliguri</t>
+          <t>Jodhpur</t>
         </is>
       </c>
     </row>
@@ -2654,12 +2654,12 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>AN</t>
+          <t>RJ</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Port Blair</t>
+          <t>Udaipur</t>
         </is>
       </c>
     </row>
@@ -2671,12 +2671,12 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>CH</t>
+          <t>RJ</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Chandigarh</t>
+          <t>Kota</t>
         </is>
       </c>
     </row>
@@ -2688,12 +2688,12 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>DH</t>
+          <t>RJ</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Daman</t>
+          <t>Ajmer</t>
         </is>
       </c>
     </row>
@@ -2705,12 +2705,12 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>DH</t>
+          <t>SK</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Silvassa</t>
+          <t>Gangtok</t>
         </is>
       </c>
     </row>
@@ -2722,12 +2722,12 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>DL</t>
+          <t>SK</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>New Delhi</t>
+          <t>Namchi</t>
         </is>
       </c>
     </row>
@@ -2739,12 +2739,12 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>DL</t>
+          <t>SK</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Delhi</t>
+          <t>Gyalshing</t>
         </is>
       </c>
     </row>
@@ -2756,12 +2756,12 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>JK</t>
+          <t>TN</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Srinagar</t>
+          <t>Chennai</t>
         </is>
       </c>
     </row>
@@ -2773,12 +2773,12 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>JK</t>
+          <t>TN</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>Jammu</t>
+          <t>Coimbatore</t>
         </is>
       </c>
     </row>
@@ -2790,12 +2790,12 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>LA</t>
+          <t>TN</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>Leh</t>
+          <t>Madurai</t>
         </is>
       </c>
     </row>
@@ -2807,12 +2807,12 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>LA</t>
+          <t>TN</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Kargil</t>
+          <t>Salem</t>
         </is>
       </c>
     </row>
@@ -2824,12 +2824,12 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>LD</t>
+          <t>TN</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Kavaratti</t>
+          <t>Tiruchirappalli</t>
         </is>
       </c>
     </row>
@@ -2841,12 +2841,12 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>PY</t>
+          <t>TS</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>Puducherry</t>
+          <t>Hyderabad</t>
         </is>
       </c>
     </row>
@@ -2858,12 +2858,590 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
+          <t>TS</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>Warangal</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>TS</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>Nizamabad</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>TS</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>Karimnagar</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>TR</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>Agartala</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>TR</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>Udaipur</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>TR</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>Dharmanagar</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>Lucknow</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>Kanpur</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>Varanasi</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>Agra</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>Prayagraj</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>Noida</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>Ghaziabad</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>Dehradun</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>Haridwar</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>Haldwani</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>Roorkee</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>WB</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>Kolkata</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>WB</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>Howrah</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>WB</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>Durgapur</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>WB</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>Siliguri</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>WB</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>Asansol</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>AN</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>Port Blair</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>Chandigarh</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>DL</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>New Delhi</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>DL</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>JK</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>Srinagar</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>JK</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>Jammu</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>LA</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>Leh</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>LA</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>Kargil</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>LD</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>Kavaratti</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
           <t>PY</t>
         </is>
       </c>
-      <c r="C104" t="inlineStr">
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>Puducherry</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>PY</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
         <is>
           <t>Karaikal</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>PY</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>Mahe</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>PY</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>Yanam</t>
         </is>
       </c>
     </row>

</xml_diff>